<commit_message>
Ajoute lastUpdated à identityReliability et affine validationDate
Ajoute une sous-extension lastUpdated (dateTime, 1..1) permettant
d'horodater et d'ordonner un historique de plusieurs instances de
l'extension identityReliability sur une même ressource, et met à
jour les exemples INS en conséquence. Précise également le libellé
de validationDate.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 22b8269fffa724bdefdfc52df4643434294856ea
</commit_message>
<xml_diff>
--- a/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
+++ b/fix/issue-298-identity-status-rniv/ig/StructureDefinition-fr-core-identity-reliability.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1370" uniqueCount="177">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-09-28T13:01:57+00:00</t>
+    <t>2026-09-28T14:15:25+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -297,21 +297,11 @@
     <t>Extension.extension</t>
   </si>
   <si>
-    <t>extensions
-user content</t>
-  </si>
-  <si>
     <t xml:space="preserve">Extension
 </t>
   </si>
   <si>
-    <t>Additional content defined by implementations</t>
-  </si>
-  <si>
-    <t>May be used to represent additional information that is not part of the basic definition of the element. To make the use of extensions safe and manageable, there is a strict set of governance  applied to the definition and use of extensions. Though any implementer can define an extension, there is a set of requirements that SHALL be met as part of the definition of the extension.</t>
-  </si>
-  <si>
-    <t>There can be no stigma associated with the use of extensions by any application, project, or standard - regardless of the institution or jurisdiction that uses or defines the extensions.  The use of extensions is what allows the FHIR specification to retain a core level of simplicity for everyone.</t>
+    <t>An Extension</t>
   </si>
   <si>
     <t xml:space="preserve">value:url}
@@ -331,34 +321,31 @@
 ext-1:Must have either extensions or value[x], not both {extension.exists() != value.exists()}</t>
   </si>
   <si>
-    <t>Extension.extension:methodCollection</t>
-  </si>
-  <si>
-    <t>methodCollection</t>
-  </si>
-  <si>
-    <t>Canal d'obtention des traits d'identité (SM, CV, INSi, CB, RFID, AV) | Channel used to collect the identity traits</t>
-  </si>
-  <si>
-    <t>Précise le canal par lequel les traits d'identité ou le matricule INS ont été obtenus : saisie manuelle, lecture de la carte Vitale, interrogation directe du téléservice INSi, scan d'un code à barre/Datamatrix, lecture RFID ou Application carte Vitale. Ce champ ne porte pas le statut de confiance résultant (cf. sous-extension `identityStatus`) ni la pièce justificative contrôlée (cf. sous-extension `validationMode`).</t>
-  </si>
-  <si>
-    <t>Extension.extension:methodCollection.id</t>
+    <t>Extension.extension:lastUpdated</t>
+  </si>
+  <si>
+    <t>lastUpdated</t>
+  </si>
+  <si>
+    <t>Date de dernière mise à jour de cette instance de l'extension, permettant d'ordonner un historique de plusieurs instances de identityReliability sur une même ressource | Date of the last update of this extension instance, used to order the history when several identityReliability instances are present on the same resource</t>
+  </si>
+  <si>
+    <t>Horodatage de la dernière mise à jour de cette instance de l'extension composite identityReliability. Dès lors que plusieurs instances de l'extension identityReliability coexistent sur la même ressource (afin de conserver un historique des statuts de confiance successifs), ce champ permet de les ordonner chronologiquement. | Timestamp of the last update of this identityReliability composite extension instance. When several identityReliability instances coexist on the same resource (to keep a history of successive trust statuses), this field allows them to be ordered chronologically.</t>
+  </si>
+  <si>
+    <t>Extension.extension:lastUpdated.id</t>
   </si>
   <si>
     <t>Extension.extension.id</t>
   </si>
   <si>
-    <t>Extension.extension:methodCollection.extension</t>
+    <t>Extension.extension:lastUpdated.extension</t>
   </si>
   <si>
     <t>Extension.extension.extension</t>
   </si>
   <si>
-    <t>An Extension</t>
-  </si>
-  <si>
-    <t>Extension.extension:methodCollection.url</t>
+    <t>Extension.extension:lastUpdated.url</t>
   </si>
   <si>
     <t>Extension.extension.url</t>
@@ -383,33 +370,61 @@
     <t>N/A</t>
   </si>
   <si>
+    <t>Extension.extension:lastUpdated.value[x]</t>
+  </si>
+  <si>
+    <t>Extension.extension.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dateTime
+</t>
+  </si>
+  <si>
+    <t>Value of extension</t>
+  </si>
+  <si>
+    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
+  </si>
+  <si>
+    <t>Extension.value[x]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+</t>
+  </si>
+  <si>
+    <t>Extension.extension:methodCollection</t>
+  </si>
+  <si>
+    <t>methodCollection</t>
+  </si>
+  <si>
+    <t>Canal d'obtention des traits d'identité (SM, CV, INSi, CB, RFID, AV) | Channel used to collect the identity traits</t>
+  </si>
+  <si>
+    <t>Précise le canal par lequel les traits d'identité ou le matricule INS ont été obtenus : saisie manuelle, lecture de la carte Vitale, interrogation directe du téléservice INSi, scan d'un code à barre/Datamatrix, lecture RFID ou Application carte Vitale. Ce champ ne porte pas le statut de confiance résultant (cf. sous-extension `identityStatus`) ni la pièce justificative contrôlée (cf. sous-extension `validationMode`).</t>
+  </si>
+  <si>
+    <t>Extension.extension:methodCollection.id</t>
+  </si>
+  <si>
+    <t>Extension.extension:methodCollection.extension</t>
+  </si>
+  <si>
+    <t>Extension.extension:methodCollection.url</t>
+  </si>
+  <si>
     <t>Extension.extension:methodCollection.value[x]</t>
-  </si>
-  <si>
-    <t>Extension.extension.value[x]</t>
   </si>
   <si>
     <t xml:space="preserve">Coding
 </t>
   </si>
   <si>
-    <t>Value of extension</t>
-  </si>
-  <si>
-    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
-  </si>
-  <si>
     <t>extensible</t>
   </si>
   <si>
     <t>https://hl7.fr/ig/fhir/core/ValueSet/fr-core-vs-identity-method-collection|2.2.0</t>
-  </si>
-  <si>
-    <t>Extension.value[x]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
-</t>
   </si>
   <si>
     <t>Extension.extension:dateInterrogationINSi</t>
@@ -501,7 +516,7 @@
     <t>validationDate</t>
   </si>
   <si>
-    <t>Date de vérification de l'identité | Identity verification date</t>
+    <t>Date du contrôle de cohérence à partir des traits portés par un dispositif d'identification à haut niveau de confiance | Date of the consistency check performed against the identity traits carried by a high-level-of-confidence identification device</t>
   </si>
   <si>
     <t>Date à laquelle l'identité a été vérifiée sur la base de la pièce justificative contrôlée (cf. sous-extension `validationMode`). | Date at which the identity was verified based on the checked supporting document (see the `validationMode` sub-extension).</t>
@@ -864,13 +879,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK36"/>
+  <dimension ref="A1:AK41"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="42.40625" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="24.9921875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="17.78125" customWidth="true" bestFit="true" hidden="true"/>
-    <col min="4" max="4" width="10.83984375" customWidth="true" bestFit="true" hidden="true"/>
+    <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
     <col min="5" max="5" width="5.80859375" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="4.23828125" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="4.65625" customWidth="true" bestFit="true"/>
@@ -1233,11 +1248,11 @@
       </c>
       <c r="C4" s="2"/>
       <c r="D4" t="s" s="2">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="E4" s="2"/>
       <c r="F4" t="s" s="2">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G4" t="s" s="2">
         <v>80</v>
@@ -1252,17 +1267,15 @@
         <v>78</v>
       </c>
       <c r="K4" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="L4" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="M4" t="s" s="2">
         <v>93</v>
       </c>
-      <c r="L4" t="s" s="2">
-        <v>94</v>
-      </c>
-      <c r="M4" t="s" s="2">
-        <v>95</v>
-      </c>
-      <c r="N4" t="s" s="2">
-        <v>96</v>
-      </c>
+      <c r="N4" s="2"/>
       <c r="O4" s="2"/>
       <c r="P4" t="s" s="2">
         <v>78</v>
@@ -1299,19 +1312,19 @@
         <v>78</v>
       </c>
       <c r="AB4" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AC4" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AD4" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE4" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AF4" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="AC4" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="AD4" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE4" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AF4" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AG4" t="s" s="2">
         <v>79</v>
@@ -1323,28 +1336,28 @@
         <v>78</v>
       </c>
       <c r="AJ4" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK4" t="s" s="2">
-        <v>90</v>
+        <v>78</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="2">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B5" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C5" t="s" s="2">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D5" t="s" s="2">
         <v>78</v>
       </c>
       <c r="E5" s="2"/>
       <c r="F5" t="s" s="2">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="G5" t="s" s="2">
         <v>85</v>
@@ -1359,13 +1372,13 @@
         <v>78</v>
       </c>
       <c r="K5" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L5" t="s" s="2">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="M5" t="s" s="2">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -1416,7 +1429,7 @@
         <v>78</v>
       </c>
       <c r="AF5" t="s" s="2">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="AG5" t="s" s="2">
         <v>79</v>
@@ -1428,7 +1441,7 @@
         <v>78</v>
       </c>
       <c r="AJ5" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK5" t="s" s="2">
         <v>78</v>
@@ -1436,10 +1449,10 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="2">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B6" t="s" s="2">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" t="s" s="2">
@@ -1539,10 +1552,10 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="2">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B7" t="s" s="2">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" t="s" s="2">
@@ -1565,13 +1578,13 @@
         <v>78</v>
       </c>
       <c r="K7" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L7" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M7" t="s" s="2">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -1610,19 +1623,19 @@
         <v>78</v>
       </c>
       <c r="AB7" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AC7" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AD7" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE7" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AF7" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="AC7" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="AD7" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE7" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AF7" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AG7" t="s" s="2">
         <v>79</v>
@@ -1634,7 +1647,7 @@
         <v>78</v>
       </c>
       <c r="AJ7" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK7" t="s" s="2">
         <v>78</v>
@@ -1642,10 +1655,10 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B8" t="s" s="2">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" t="s" s="2">
@@ -1668,16 +1681,16 @@
         <v>78</v>
       </c>
       <c r="K8" t="s" s="2">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="L8" t="s" s="2">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="M8" t="s" s="2">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="N8" t="s" s="2">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="O8" s="2"/>
       <c r="P8" t="s" s="2">
@@ -1685,7 +1698,7 @@
       </c>
       <c r="Q8" s="2"/>
       <c r="R8" t="s" s="2">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="S8" t="s" s="2">
         <v>78</v>
@@ -1727,7 +1740,7 @@
         <v>78</v>
       </c>
       <c r="AF8" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="AG8" t="s" s="2">
         <v>85</v>
@@ -1742,15 +1755,15 @@
         <v>78</v>
       </c>
       <c r="AK8" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B9" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" t="s" s="2">
@@ -1773,13 +1786,13 @@
         <v>78</v>
       </c>
       <c r="K9" t="s" s="2">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="L9" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="M9" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -1806,11 +1819,13 @@
         <v>78</v>
       </c>
       <c r="X9" t="s" s="2">
-        <v>124</v>
-      </c>
-      <c r="Y9" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="Y9" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="Z9" t="s" s="2">
-        <v>125</v>
+        <v>78</v>
       </c>
       <c r="AA9" t="s" s="2">
         <v>78</v>
@@ -1828,7 +1843,7 @@
         <v>78</v>
       </c>
       <c r="AF9" t="s" s="2">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="AG9" t="s" s="2">
         <v>79</v>
@@ -1840,21 +1855,21 @@
         <v>78</v>
       </c>
       <c r="AJ9" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="AK9" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="2">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="B10" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C10" t="s" s="2">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="D10" t="s" s="2">
         <v>78</v>
@@ -1876,13 +1891,13 @@
         <v>78</v>
       </c>
       <c r="K10" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -1933,7 +1948,7 @@
         <v>78</v>
       </c>
       <c r="AF10" t="s" s="2">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="AG10" t="s" s="2">
         <v>79</v>
@@ -1945,7 +1960,7 @@
         <v>78</v>
       </c>
       <c r="AJ10" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK10" t="s" s="2">
         <v>78</v>
@@ -1953,10 +1968,10 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
@@ -2056,10 +2071,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2082,13 +2097,13 @@
         <v>78</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L12" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2127,19 +2142,19 @@
         <v>78</v>
       </c>
       <c r="AB12" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AC12" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AD12" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE12" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AF12" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="AC12" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="AD12" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE12" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AF12" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>79</v>
@@ -2151,7 +2166,7 @@
         <v>78</v>
       </c>
       <c r="AJ12" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK12" t="s" s="2">
         <v>78</v>
@@ -2159,10 +2174,10 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2185,16 +2200,16 @@
         <v>78</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" t="s" s="2">
@@ -2202,7 +2217,7 @@
       </c>
       <c r="Q13" s="2"/>
       <c r="R13" t="s" s="2">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="S13" t="s" s="2">
         <v>78</v>
@@ -2244,7 +2259,7 @@
         <v>78</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>85</v>
@@ -2259,15 +2274,15 @@
         <v>78</v>
       </c>
       <c r="AK13" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -2290,13 +2305,13 @@
         <v>78</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2323,13 +2338,11 @@
         <v>78</v>
       </c>
       <c r="X14" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y14" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="Y14" s="2"/>
       <c r="Z14" t="s" s="2">
-        <v>78</v>
+        <v>132</v>
       </c>
       <c r="AA14" t="s" s="2">
         <v>78</v>
@@ -2347,7 +2360,7 @@
         <v>78</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>79</v>
@@ -2359,21 +2372,21 @@
         <v>78</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="AK14" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="B15" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>78</v>
@@ -2395,13 +2408,13 @@
         <v>78</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>110</v>
+        <v>136</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2452,7 +2465,7 @@
         <v>78</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>79</v>
@@ -2464,7 +2477,7 @@
         <v>78</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK15" t="s" s="2">
         <v>78</v>
@@ -2472,10 +2485,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -2575,10 +2588,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -2601,13 +2614,13 @@
         <v>78</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L17" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="N17" s="2"/>
       <c r="O17" s="2"/>
@@ -2646,19 +2659,19 @@
         <v>78</v>
       </c>
       <c r="AB17" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AF17" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>79</v>
@@ -2670,7 +2683,7 @@
         <v>78</v>
       </c>
       <c r="AJ17" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK17" t="s" s="2">
         <v>78</v>
@@ -2678,10 +2691,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -2704,16 +2717,16 @@
         <v>78</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -2721,7 +2734,7 @@
       </c>
       <c r="Q18" s="2"/>
       <c r="R18" t="s" s="2">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="S18" t="s" s="2">
         <v>78</v>
@@ -2763,7 +2776,7 @@
         <v>78</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>85</v>
@@ -2778,15 +2791,15 @@
         <v>78</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -2809,13 +2822,13 @@
         <v>78</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -2842,11 +2855,13 @@
         <v>78</v>
       </c>
       <c r="X19" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="Y19" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="Y19" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="Z19" t="s" s="2">
-        <v>145</v>
+        <v>78</v>
       </c>
       <c r="AA19" t="s" s="2">
         <v>78</v>
@@ -2864,7 +2879,7 @@
         <v>78</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>79</v>
@@ -2876,21 +2891,21 @@
         <v>78</v>
       </c>
       <c r="AJ19" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="AK19" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B20" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C20" t="s" s="2">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="D20" t="s" s="2">
         <v>78</v>
@@ -2900,7 +2915,7 @@
         <v>79</v>
       </c>
       <c r="G20" t="s" s="2">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="H20" t="s" s="2">
         <v>78</v>
@@ -2912,13 +2927,13 @@
         <v>78</v>
       </c>
       <c r="K20" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="L20" t="s" s="2">
+        <v>144</v>
+      </c>
+      <c r="M20" t="s" s="2">
         <v>93</v>
-      </c>
-      <c r="L20" t="s" s="2">
-        <v>148</v>
-      </c>
-      <c r="M20" t="s" s="2">
-        <v>110</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -2969,7 +2984,7 @@
         <v>78</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>79</v>
@@ -2981,7 +2996,7 @@
         <v>78</v>
       </c>
       <c r="AJ20" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK20" t="s" s="2">
         <v>78</v>
@@ -2989,10 +3004,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3092,10 +3107,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3118,13 +3133,13 @@
         <v>78</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L22" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3163,19 +3178,19 @@
         <v>78</v>
       </c>
       <c r="AB22" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AC22" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AD22" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE22" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AF22" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="AC22" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="AD22" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE22" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AF22" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
@@ -3187,7 +3202,7 @@
         <v>78</v>
       </c>
       <c r="AJ22" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK22" t="s" s="2">
         <v>78</v>
@@ -3195,10 +3210,10 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
@@ -3221,16 +3236,16 @@
         <v>78</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -3238,7 +3253,7 @@
       </c>
       <c r="Q23" s="2"/>
       <c r="R23" t="s" s="2">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="S23" t="s" s="2">
         <v>78</v>
@@ -3280,7 +3295,7 @@
         <v>78</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>85</v>
@@ -3295,15 +3310,15 @@
         <v>78</v>
       </c>
       <c r="AK23" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3326,13 +3341,13 @@
         <v>78</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>153</v>
+        <v>130</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3359,11 +3374,11 @@
         <v>78</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>124</v>
+        <v>149</v>
       </c>
       <c r="Y24" s="2"/>
       <c r="Z24" t="s" s="2">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>78</v>
@@ -3381,7 +3396,7 @@
         <v>78</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>79</v>
@@ -3393,21 +3408,21 @@
         <v>78</v>
       </c>
       <c r="AJ24" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="AK24" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>155</v>
+        <v>151</v>
       </c>
       <c r="B25" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C25" t="s" s="2">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="D25" t="s" s="2">
         <v>78</v>
@@ -3417,7 +3432,7 @@
         <v>79</v>
       </c>
       <c r="G25" t="s" s="2">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="H25" t="s" s="2">
         <v>78</v>
@@ -3429,13 +3444,13 @@
         <v>78</v>
       </c>
       <c r="K25" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="L25" t="s" s="2">
+        <v>153</v>
+      </c>
+      <c r="M25" t="s" s="2">
         <v>93</v>
-      </c>
-      <c r="L25" t="s" s="2">
-        <v>157</v>
-      </c>
-      <c r="M25" t="s" s="2">
-        <v>158</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -3486,7 +3501,7 @@
         <v>78</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
@@ -3498,7 +3513,7 @@
         <v>78</v>
       </c>
       <c r="AJ25" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK25" t="s" s="2">
         <v>78</v>
@@ -3506,10 +3521,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -3609,10 +3624,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -3635,13 +3650,13 @@
         <v>78</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L27" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -3680,19 +3695,19 @@
         <v>78</v>
       </c>
       <c r="AB27" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AC27" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AD27" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE27" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AF27" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="AC27" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="AD27" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE27" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AF27" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>79</v>
@@ -3704,7 +3719,7 @@
         <v>78</v>
       </c>
       <c r="AJ27" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK27" t="s" s="2">
         <v>78</v>
@@ -3712,10 +3727,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -3738,16 +3753,16 @@
         <v>78</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -3755,7 +3770,7 @@
       </c>
       <c r="Q28" s="2"/>
       <c r="R28" t="s" s="2">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="S28" t="s" s="2">
         <v>78</v>
@@ -3797,7 +3812,7 @@
         <v>78</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>85</v>
@@ -3812,15 +3827,15 @@
         <v>78</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -3843,13 +3858,13 @@
         <v>78</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -3876,13 +3891,11 @@
         <v>78</v>
       </c>
       <c r="X29" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="Y29" t="s" s="2">
-        <v>78</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="Y29" s="2"/>
       <c r="Z29" t="s" s="2">
-        <v>78</v>
+        <v>159</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>78</v>
@@ -3900,7 +3913,7 @@
         <v>78</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>79</v>
@@ -3912,21 +3925,21 @@
         <v>78</v>
       </c>
       <c r="AJ29" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B30" t="s" s="2">
         <v>91</v>
       </c>
       <c r="C30" t="s" s="2">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="D30" t="s" s="2">
         <v>78</v>
@@ -3948,13 +3961,13 @@
         <v>78</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>110</v>
+        <v>163</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" s="2"/>
@@ -4005,7 +4018,7 @@
         <v>78</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>79</v>
@@ -4017,7 +4030,7 @@
         <v>78</v>
       </c>
       <c r="AJ30" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK30" t="s" s="2">
         <v>78</v>
@@ -4025,10 +4038,10 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
@@ -4128,10 +4141,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -4154,13 +4167,13 @@
         <v>78</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="L32" t="s" s="2">
         <v>32</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>110</v>
+        <v>93</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -4199,19 +4212,19 @@
         <v>78</v>
       </c>
       <c r="AB32" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AC32" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AD32" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE32" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AF32" t="s" s="2">
         <v>97</v>
-      </c>
-      <c r="AC32" t="s" s="2">
-        <v>98</v>
-      </c>
-      <c r="AD32" t="s" s="2">
-        <v>78</v>
-      </c>
-      <c r="AE32" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="AF32" t="s" s="2">
-        <v>100</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>79</v>
@@ -4223,7 +4236,7 @@
         <v>78</v>
       </c>
       <c r="AJ32" t="s" s="2">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="AK32" t="s" s="2">
         <v>78</v>
@@ -4231,10 +4244,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -4257,16 +4270,16 @@
         <v>78</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="N33" t="s" s="2">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="O33" s="2"/>
       <c r="P33" t="s" s="2">
@@ -4274,7 +4287,7 @@
       </c>
       <c r="Q33" s="2"/>
       <c r="R33" t="s" s="2">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="S33" t="s" s="2">
         <v>78</v>
@@ -4316,7 +4329,7 @@
         <v>78</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>85</v>
@@ -4331,15 +4344,15 @@
         <v>78</v>
       </c>
       <c r="AK33" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -4362,13 +4375,13 @@
         <v>78</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>121</v>
+        <v>141</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -4395,11 +4408,13 @@
         <v>78</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>144</v>
-      </c>
-      <c r="Y34" s="2"/>
+        <v>78</v>
+      </c>
+      <c r="Y34" t="s" s="2">
+        <v>78</v>
+      </c>
       <c r="Z34" t="s" s="2">
-        <v>170</v>
+        <v>78</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>78</v>
@@ -4417,7 +4432,7 @@
         <v>78</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>126</v>
+        <v>120</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -4429,26 +4444,28 @@
         <v>78</v>
       </c>
       <c r="AJ34" t="s" s="2">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="AK34" t="s" s="2">
-        <v>118</v>
+        <v>114</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>117</v>
+        <v>168</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>117</v>
-      </c>
-      <c r="C35" s="2"/>
+        <v>91</v>
+      </c>
+      <c r="C35" t="s" s="2">
+        <v>169</v>
+      </c>
       <c r="D35" t="s" s="2">
         <v>78</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="G35" t="s" s="2">
         <v>85</v>
@@ -4463,24 +4480,22 @@
         <v>78</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>113</v>
+        <v>92</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>114</v>
+        <v>170</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>115</v>
-      </c>
-      <c r="N35" t="s" s="2">
-        <v>116</v>
-      </c>
+        <v>93</v>
+      </c>
+      <c r="N35" s="2"/>
       <c r="O35" s="2"/>
       <c r="P35" t="s" s="2">
         <v>78</v>
       </c>
       <c r="Q35" s="2"/>
       <c r="R35" t="s" s="2">
-        <v>3</v>
+        <v>78</v>
       </c>
       <c r="S35" t="s" s="2">
         <v>78</v>
@@ -4522,30 +4537,30 @@
         <v>78</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>117</v>
+        <v>97</v>
       </c>
       <c r="AG35" t="s" s="2">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="AI35" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AJ35" t="s" s="2">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="AK35" t="s" s="2">
-        <v>118</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>126</v>
+        <v>171</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -4556,7 +4571,7 @@
         <v>79</v>
       </c>
       <c r="G36" t="s" s="2">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="H36" t="s" s="2">
         <v>78</v>
@@ -4568,13 +4583,13 @@
         <v>78</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>171</v>
+        <v>86</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>122</v>
+        <v>87</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>123</v>
+        <v>88</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -4625,7 +4640,7 @@
         <v>78</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>126</v>
+        <v>89</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
@@ -4637,10 +4652,527 @@
         <v>78</v>
       </c>
       <c r="AJ36" t="s" s="2">
-        <v>127</v>
+        <v>78</v>
       </c>
       <c r="AK36" t="s" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s" s="2">
+        <v>172</v>
+      </c>
+      <c r="B37" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E37" s="2"/>
+      <c r="F37" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G37" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K37" t="s" s="2">
+        <v>92</v>
+      </c>
+      <c r="L37" t="s" s="2">
+        <v>32</v>
+      </c>
+      <c r="M37" t="s" s="2">
+        <v>93</v>
+      </c>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q37" s="2"/>
+      <c r="R37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB37" t="s" s="2">
+        <v>94</v>
+      </c>
+      <c r="AC37" t="s" s="2">
+        <v>95</v>
+      </c>
+      <c r="AD37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE37" t="s" s="2">
+        <v>96</v>
+      </c>
+      <c r="AF37" t="s" s="2">
+        <v>97</v>
+      </c>
+      <c r="AG37" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH37" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="AI37" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ37" t="s" s="2">
+        <v>98</v>
+      </c>
+      <c r="AK37" t="s" s="2">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s" s="2">
+        <v>173</v>
+      </c>
+      <c r="B38" t="s" s="2">
+        <v>108</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E38" s="2"/>
+      <c r="F38" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="G38" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K38" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="L38" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="M38" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="N38" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="O38" s="2"/>
+      <c r="P38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q38" s="2"/>
+      <c r="R38" t="s" s="2">
+        <v>169</v>
+      </c>
+      <c r="S38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF38" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="AG38" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH38" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ38" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK38" t="s" s="2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s" s="2">
+        <v>174</v>
+      </c>
+      <c r="B39" t="s" s="2">
+        <v>116</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E39" s="2"/>
+      <c r="F39" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G39" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K39" t="s" s="2">
+        <v>130</v>
+      </c>
+      <c r="L39" t="s" s="2">
         <v>118</v>
+      </c>
+      <c r="M39" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
+      <c r="P39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q39" s="2"/>
+      <c r="R39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X39" t="s" s="2">
+        <v>149</v>
+      </c>
+      <c r="Y39" s="2"/>
+      <c r="Z39" t="s" s="2">
+        <v>175</v>
+      </c>
+      <c r="AA39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF39" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="AG39" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH39" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI39" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ39" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="AK39" t="s" s="2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="B40" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E40" s="2"/>
+      <c r="F40" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="G40" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K40" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="L40" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="M40" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="N40" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="O40" s="2"/>
+      <c r="P40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q40" s="2"/>
+      <c r="R40" t="s" s="2">
+        <v>3</v>
+      </c>
+      <c r="S40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF40" t="s" s="2">
+        <v>113</v>
+      </c>
+      <c r="AG40" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AH40" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ40" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AK40" t="s" s="2">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="B41" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="E41" s="2"/>
+      <c r="F41" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="G41" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="H41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="I41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="J41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="K41" t="s" s="2">
+        <v>176</v>
+      </c>
+      <c r="L41" t="s" s="2">
+        <v>118</v>
+      </c>
+      <c r="M41" t="s" s="2">
+        <v>119</v>
+      </c>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2"/>
+      <c r="P41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Q41" s="2"/>
+      <c r="R41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="S41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="T41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="U41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="V41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="W41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="X41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Y41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="Z41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AA41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AB41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AC41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AD41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AE41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AF41" t="s" s="2">
+        <v>120</v>
+      </c>
+      <c r="AG41" t="s" s="2">
+        <v>79</v>
+      </c>
+      <c r="AH41" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI41" t="s" s="2">
+        <v>78</v>
+      </c>
+      <c r="AJ41" t="s" s="2">
+        <v>121</v>
+      </c>
+      <c r="AK41" t="s" s="2">
+        <v>114</v>
       </c>
     </row>
   </sheetData>

</xml_diff>